<commit_message>
Add README, Result and update bug reports
</commit_message>
<xml_diff>
--- a/Bug_reports.xlsx
+++ b/Bug_reports.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Баг-репорты" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Баг-репорты'!$A$1:$L$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Баг-репорты'!$A$1:$M$13</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -452,7 +452,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L13"/>
+  <dimension ref="A1:M13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -467,6 +467,7 @@
     <col width="16" customWidth="1" min="10" max="10"/>
     <col width="40" customWidth="1" min="11" max="11"/>
     <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="70" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -530,6 +531,11 @@
           <t>Статус</t>
         </is>
       </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Дополнительная информация</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -592,6 +598,11 @@
           <t>Открыт</t>
         </is>
       </c>
+      <c r="M2" s="3" t="inlineStr">
+        <is>
+          <t>Анализ исходного кода подтверждает, что корректное сообщение предусмотрено разработчиками, но недостижимо. В app/src/main/res/values/strings.xml присутствует строка wrong_login_or_password со значением Wrong login or password. В AuthFragment реализован обработчик события authorizationFailedExceptionEvent, который выводит именно эту строку. Однако при вводе неверных учётных данных срабатывает обработчик события loginExceptionEvent, показывающий общее сообщение из строки error. Ошибка авторизации не выделяется в отдельное событие и обрабатывается наравне с прочими сбоями.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -654,6 +665,7 @@
           <t>Открыт</t>
         </is>
       </c>
+      <c r="M3" s="3" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -716,6 +728,7 @@
           <t>Открыт</t>
         </is>
       </c>
+      <c r="M4" s="3" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -778,6 +791,7 @@
           <t>Открыт</t>
         </is>
       </c>
+      <c r="M5" s="3" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -840,6 +854,11 @@
           <t>Открыт</t>
         </is>
       </c>
+      <c r="M6" s="3" t="inlineStr">
+        <is>
+          <t>Поле Creation date заполняется приложением автоматически и не доступно для ввода пользователем. Значение поля Publication date при этом отображается корректно, что указывает на дефект обработки конкретного значения, а не на ошибку ввода.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -902,6 +921,7 @@
           <t>Открыт</t>
         </is>
       </c>
+      <c r="M7" s="3" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -964,6 +984,7 @@
           <t>Открыт</t>
         </is>
       </c>
+      <c r="M8" s="3" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1026,6 +1047,7 @@
           <t>Открыт</t>
         </is>
       </c>
+      <c r="M9" s="3" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1088,6 +1110,7 @@
           <t>Открыт</t>
         </is>
       </c>
+      <c r="M10" s="3" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1150,6 +1173,7 @@
           <t>Открыт</t>
         </is>
       </c>
+      <c r="M11" s="3" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1212,6 +1236,11 @@
           <t>Открыт</t>
         </is>
       </c>
+      <c r="M12" s="3" t="inlineStr">
+        <is>
+          <t>Состояние элемента подтверждено данными системы. В иерархии элементов интерфейса, полученной при выполнении автотеста на экране News, пункт меню About имеет атрибут is-enabled=false, тогда как пункты Main и News — is-enabled=true. Пункт меню программно отключён, а не просто не реагирует на нажатие.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1274,9 +1303,10 @@
           <t>Открыт</t>
         </is>
       </c>
+      <c r="M13" s="3" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L13"/>
+  <autoFilter ref="A1:M13"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>